<commit_message>
Update: office 35만원 + room 70만원 + deposit 100만원
</commit_message>
<xml_diff>
--- a/files/ResonateClub_5천만원_창업비용_분석.xlsx
+++ b/files/ResonateClub_5천만원_창업비용_분석.xlsx
@@ -176,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -212,6 +212,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -228,9 +234,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -238,7 +241,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -612,25 +615,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RESONATE CLUB — 국내외여행업 1인 주식회사 창업 비용 분석</t>
+          <t>RESONATE CLUB — 국내외여행업 1인 주식회사 창업 비용</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>작성일: 2026년 5월 26일 | 자본금: 5,000만원 | F-4 비자</t>
+          <t>작성일: 2026.05.26 | 자본금: 5,000만원 | F-4 비자 | 해운대</t>
         </is>
       </c>
     </row>
@@ -673,161 +676,178 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>10000000</v>
+        <v>1000000</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>해운대 소형 오피스, 초기 1회, 퇴거 시 반환</t>
+          <t>월세 35만원 오피스, 초기 1회, 퇴거 시 반환</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>📋 법인설립 등기비</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>400000</v>
+          <t>🏠 주거 보증금</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>무료</t>
+        </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>전자등기 수수료 + 등록면허세</t>
+          <t>방세 70만원 — 보증금 포함 가정</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>📋 사업자등록</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>무료</t>
-        </is>
+          <t>📋 법인설립 등기비</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>400000</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>무료, 세무서 방문</t>
+          <t>전자등기 수수료 + 등록면허세</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>📋 여행업 등록 수수료</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>50000</v>
+          <t>📋 사업자등록</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>무료</t>
+        </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>해운대구청</t>
+          <t>무료, 해운대세무서</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>🛡️ 영업보증보험 (1년)</t>
+          <t>📋 여행업 등록 수수료</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>1000000</v>
+        <v>50000</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>5천만원 보증, 연 0.5~1% 요율</t>
+          <t>해운대구청</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>🪑 사무실 초도 비품</t>
+          <t>🛡️ 영업보증보험 (1년)</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>책상, 의자, 컴퓨터, 프린터 등</t>
+          <t>5천만원 보증, 연 0.5~1% 요율</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>🌐 웹사이트 도메인 (1년)</t>
+          <t>🪑 사무실 초도 비품</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>50000</v>
+        <v>2000000</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>resonateclub.com, resonatetour.com</t>
+          <t>책상, 의자, 컴퓨터, 프린터 등</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>📞 통신 개통비</t>
+          <t>🌐 웹사이트·도메인 (1년)</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>인터넷 + 전화</t>
+          <t>resonateclub.com, resonatetour.com</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>📞 통신 개통비</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>인터넷 + 전화</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>📦 기타 초기 잡비</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B15" s="7" t="n">
         <v>500000</v>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>인쇄물, 명함, 소모품 등</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>📊 초기 소요 자금 (자본금 제외)</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
-        <v>14100000</v>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>실제 지출되는 현금</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>📊 자본금 포함 총 현금 확보 필요</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>64100000</v>
+      <c r="B16" s="10" t="n">
+        <v>5100000</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>실제 지출되는 현금 (사무실 보증금 포함)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>📊 자본금 포함 총 현금</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>55100000</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>통장 잔고 증빙 + 실제 초기 지출</t>
         </is>
@@ -849,19 +869,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>월 고정비 상세 (국내외여행업 1인 주식회사)</t>
+          <t>월 고정비 상세</t>
         </is>
       </c>
     </row>
@@ -890,79 +910,79 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>🏢 사무실 임대 (해운대)</t>
+          <t>🏢 사무실 월세 (해운대)</t>
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>800000</v>
+        <v>350000</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>9600000</v>
+        <v>4200000</v>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>월 100만원 → 20% 절감 협상 적용</t>
+          <t>소형 오피스, 월 35만원</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>🛡️ 영업보증보험료</t>
+          <t>🏠 방세 (주거)</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>83000</v>
+        <v>700000</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1000000</v>
+        <v>8400000</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>5천만원 보증, 연 0.5~1%, 보수적 100만원/년</t>
+          <t>1인 거주, 월 70만원</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>📊 회계·세무 대행</t>
+          <t>🛡️ 영업보증보험료</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>300000</v>
+        <v>83000</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>3600000</v>
+        <v>1000000</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>월 30만원, 1인 법인 기준</t>
+          <t>5천만원 보증, 연 0.5~1%, 보수적 100만원/년</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>📞 통신·사무용품</t>
+          <t>📊 회계·세무 대행</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>200000</v>
+        <v>300000</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>2400000</v>
+        <v>3600000</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>인터넷, 전화, 문구, 프린터 토너 등</t>
+          <t>월 30만원, 1인 법인 기준</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>🔧 기타 잡비</t>
+          <t>📞 통신·사무용품</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
@@ -973,25 +993,25 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>경조사비, 비정기 소모품, 소프트웨어 등</t>
+          <t>인터넷, 전화, 문구, 토너 등</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>📦 예비비 (운전자본)</t>
+          <t>🔧 기타 잡비</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0</v>
+        <v>2400000</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>별도 통장 500만원 유지 권장, 월 고정비 아님</t>
+          <t>경조사비, 소모품, 소프트웨어 등</t>
         </is>
       </c>
     </row>
@@ -1002,45 +1022,56 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>1583000</v>
+        <v>1833000</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>19000000</v>
+        <v>22000000</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>연간 약 1,900만원</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+          <t>사업+주거 포함 연 약 2,200만원</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>📊 순수 사업 월 고정비</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>1133000</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>13600000</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>방세 제외, 사업만</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>📌 특이사항</t>
         </is>
       </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="15" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>• 영업보증보험: 연 15% 대출이자와 혼동 금지. 실제 보증보험 요율은 연 0.5~1%</t>
-        </is>
-      </c>
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="16" t="n"/>
+      <c r="D13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>• 예비비: 월 고정비가 아닌 별도 운전자본 500만원 통장 유지 권장</t>
+          <t>• 영업보증보험: 연 15% 대출이자와 혼동 금지. 실제 보증보험 요율은 연 0.5~1%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>• 사무실 보증금(1,000만원)은 월 비용 아님. 퇴거 시 반환</t>
+          <t>• 사무실 보증금(100만원)은 월 비용 아님. 퇴거 시 반환</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1085,14 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>• 미국 F-4 비자 대표: 외국인등록증 추가 외 모든 절차 내국인과 동일</t>
+          <t>• 방세 70만원은 주거비 — 사업 손비 처리 가능 여부 세무사 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>• F-4 비자: 외국인등록증 추가 외 모든 절차 내국인과 동일</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1100,7 @@
   <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A18:D18"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="A13:D13"/>
@@ -1088,7 +1126,7 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1136,245 +1174,245 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>법인설립등기</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>부산지방법원 / startbiz.go.kr</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>1~2주</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>~40만원</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>1~2주차</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
-        <is>
-          <t>F-4는 외국인등록번호로 온라인 신청 가능</t>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>F-4 외국인등록번호로 온라인 가능</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>사업자등록</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>해운대세무서</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>1주</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>무료</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>2~3주차</t>
         </is>
       </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>법인등기 완료 후 즉시 신청</t>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>법인등기 후 즉시</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>법인 통장 개설</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>은행</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>1일</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>무료</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>3주차</t>
         </is>
       </c>
-      <c r="G6" s="17" t="inlineStr">
+      <c r="G6" s="19" t="inlineStr">
         <is>
           <t>자본금 5천만원 예치 증빙</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>사무실 임대차 계약</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>부동산중개소</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>1주</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>보증금 1천만원</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>보증금 100만원</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>1~4주차</t>
         </is>
       </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
-          <t>법인 명의 계약 필수, 해운대구 소재</t>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>법인 명의, 해운대구 소재</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>여행업 등록 신청</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>해운대구청 문화관광과</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>2~4주</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>~5만원</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>4~8주차</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
-        <is>
-          <t>사업계획서, 자본금 증빙, 사무실 증빙, 법인등기부등본</t>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>사업계획서+자본금증빙+사무실증빙+법인등기부</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>영업보증보험 가입</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>서울보증보험 / KATA</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>1주</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>~100만원/년</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>5~8주차</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>5천만원 보증. 여행업 등록증 필요</t>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>5천만원 보증, 등록증 필요</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>관광협회 가입 (권장)</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>관광협회 가입(권장)</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>한국관광협회중앙회</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>1주</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>~20만원/년</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="18" t="inlineStr">
         <is>
           <t>8주차</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>업계 네트워크, 공제 혜택</t>
         </is>
@@ -1395,10 +1433,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -1408,7 +1446,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>1년차 현금흐름 추정 (국내외여행업, 1인)</t>
+          <t>1년차 현금흐름 추정 (보수적, 연 6팀)</t>
         </is>
       </c>
     </row>
@@ -1440,18 +1478,18 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>📈 예상 매출</t>
         </is>
       </c>
-      <c r="B4" s="14" t="n"/>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="15" t="n"/>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>한국인→미국 골프 (연 6팀)</t>
         </is>
@@ -1461,12 +1499,12 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Trump Premier $6,579 × 6팀 × ₩1,350 = 약 5,330만원</t>
+          <t>Trump Premier $6,579 × 6팀 × ₩1,350</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>소규모 맞춤 여행 (연 4건)</t>
         </is>
@@ -1486,38 +1524,38 @@
           <t>매출 합계</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="14" t="n">
         <v>51500000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>📉 비용</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="15" t="n"/>
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>월 고정비 × 12</t>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>사업 월 고정비 × 12</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>19000000</v>
+        <v>13600000</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>사무실 + 보험 + 회계 + 통신 + 잡비</t>
+          <t>사무실+보험+회계+통신+잡비 (방세 제외)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>골프장 그린피 원가 (6팀)</t>
         </is>
@@ -1527,12 +1565,12 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>팀당 약 58만원 × 6</t>
+          <t>팀당 약 58만원</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>숙박 원가 (6팀)</t>
         </is>
@@ -1542,12 +1580,12 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>팀당 약 117만원 × 6</t>
+          <t>팀당 약 117만원</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>식사 원가 (6팀)</t>
         </is>
@@ -1557,12 +1595,12 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>팀당 약 83만원 × 6</t>
+          <t>팀당 약 83만원</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>차량·가이드 원가 (6팀)</t>
         </is>
@@ -1572,22 +1610,22 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>팀당 약 133만원 × 6</t>
+          <t>팀당 약 133만원</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>초기 설립비 (1회성)</t>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>초기 설립비 감가 (1년)</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>2000000</v>
+        <v>5100000</v>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>등기·등록·비품 등 감가상각</t>
+          <t>등기·등록·비품 등</t>
         </is>
       </c>
     </row>
@@ -1598,82 +1636,74 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>44500000</v>
+        <v>42210000</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>💰 순이익 (세전)</t>
         </is>
       </c>
-      <c r="B18" s="21" t="n">
-        <v>7000000</v>
-      </c>
-      <c r="C18" s="22" t="inlineStr">
-        <is>
-          <t>13.6%</t>
-        </is>
-      </c>
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>연 6팀 기준 보수적 추정</t>
+      <c r="B18" s="22" t="n">
+        <v>9290000</v>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>18.0%</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>연 6팀 기준. 연 10팀 시 순이익 약 1,870만원</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>📌 참고</t>
         </is>
       </c>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="15" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="17" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>• 위 추정은 보수적 시나리오 (연 6팀). 팀당 순마진 약 117만원</t>
+          <t>• 위 추정은 보수적 시나리오 (연 6팀). 팀당 순마진 약 155만원</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>• 연 10팀 달성 시 순이익 약 1,700만원으로 증가</t>
+          <t>• 종합여행업 전환 시 미국인 인바운드 추가 매출 (연 2~4팀 → +2,000~5,000만원)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>• 종합여행업 전환 시 미국인 인바운드 추가 매출 가능 (연 2~4팀 → +2,000~5,000만원)</t>
+          <t>• F-4 미국인 대표: 미국 현지 직접 수배로 중간 마진 제거 → 원가 절감 가능</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>• F-4 미국인 대표: 미국 현지 직접 수배로 원가 절감 가능 (중간 유통 마진 제거)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>• 세금: 법인세 9% (과세표준 2억 이하), 부가세는 외국인 대상 영세율 적용 가능</t>
+          <t>• 세금: 법인세 9% (과세표준 2억 이하)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="8">
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A25:E25"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A22:E22"/>
@@ -1690,14 +1720,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1725,7 +1755,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>추가 필요 자금</t>
+          <t>추가 자금</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1735,208 +1765,208 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>법인 자본금 증자 (5천→1억)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>1~2주</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>~9만원</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>4,000만원</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
-        <is>
-          <t>주식 발행, 1인 주주 의사록, 변경등기</t>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>1인 주주 의사록, 변경등기</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>사업자등록 정정</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>1주</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>무료</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>0원</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>자본금 금액 변경</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>여행업 변경등록</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>2~4주</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>~5만원</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>0원</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>해운대구청, 기존 등록증 반납</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>보증보험 변경</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>1주</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>변동 미미</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>0원</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>기본 보증 동일(5천만원), 기획여행 시 추가</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>관광협회 회원 변경</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>1주</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>~5만원</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>0원</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>등급 변경 신고</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>📌 총 전환 비용 요약</t>
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>📌 총 전환 비용</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>추가 납입자본금</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>회사 통장 예치, 운영자금 사용 가능</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>추가 납입자본금</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>40000000</v>
+          <t>행정 비용</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>200000</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>회사 통장 예치, 운영자금으로 사용 가능</t>
+          <t>등기 + 등록 수수료</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>행정 비용</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>200000</v>
+          <t>총 소요 기간</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>3~4주</t>
+        </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>등기 + 등록 수수료</t>
+          <t>모든 절차 병행 가능</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>총 소요 기간</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>3~4주</t>
+          <t>전환 트리거</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>인바운드 수요 시</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>모든 절차 병행 가능</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>전환 트리거</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>인바운드 수요 확인 시</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>첫 미국인 고객 확보 1~2개월 전 시작</t>
+          <t>첫 외국인 고객 1~2개월 전 시작</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: remove transparent pricing, scope to 국내외여행업, equipment 200→100만원
</commit_message>
<xml_diff>
--- a/files/ResonateClub_5천만원_창업비용_분석.xlsx
+++ b/files/ResonateClub_5천만원_창업비용_분석.xlsx
@@ -629,6 +629,8 @@
           <t>RESONATE CLUB — 국내외여행업 1인 주식회사 창업 비용</t>
         </is>
       </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="17" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -636,6 +638,8 @@
           <t>작성일: 2026.05.26 | 자본금: 5,000만원 | F-4 비자 | 해운대</t>
         </is>
       </c>
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="17" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -770,7 +774,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
@@ -830,7 +834,7 @@
         </is>
       </c>
       <c r="B16" s="10" t="n">
-        <v>5100000</v>
+        <v>4100000</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
@@ -845,7 +849,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>55100000</v>
+        <v>54100000</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
@@ -884,6 +888,9 @@
           <t>월 고정비 상세</t>
         </is>
       </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1067,6 +1074,9 @@
           <t>• 영업보증보험: 연 15% 대출이자와 혼동 금지. 실제 보증보험 요율은 연 0.5~1%</t>
         </is>
       </c>
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="17" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1074,6 +1084,9 @@
           <t>• 사무실 보증금(100만원)은 월 비용 아님. 퇴거 시 반환</t>
         </is>
       </c>
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="17" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1081,6 +1094,9 @@
           <t>• 자본금 5,000만원은 회사 통장에 예치. 사업 운영비로 인출 사용 가능</t>
         </is>
       </c>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="17" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1088,6 +1104,9 @@
           <t>• 방세 70만원은 주거비 — 사업 손비 처리 가능 여부 세무사 확인</t>
         </is>
       </c>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1095,6 +1114,9 @@
           <t>• F-4 비자: 외국인등록증 추가 외 모든 절차 내국인과 동일</t>
         </is>
       </c>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1135,6 +1157,12 @@
           <t>절차별 소요 시간 및 비용 — 총 6~8주</t>
         </is>
       </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1449,6 +1477,10 @@
           <t>1년차 현금흐름 추정 (보수적, 연 6팀)</t>
         </is>
       </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1621,7 +1653,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>5100000</v>
+        <v>4100000</v>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
@@ -1636,7 +1668,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>42210000</v>
+        <v>41210000</v>
       </c>
     </row>
     <row r="18">
@@ -1646,11 +1678,11 @@
         </is>
       </c>
       <c r="B18" s="22" t="n">
-        <v>9290000</v>
+        <v>10290000</v>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="E18" s="24" t="inlineStr">
@@ -1676,6 +1708,10 @@
           <t>• 위 추정은 보수적 시나리오 (연 6팀). 팀당 순마진 약 155만원</t>
         </is>
       </c>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="17" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1683,6 +1719,10 @@
           <t>• 종합여행업 전환 시 미국인 인바운드 추가 매출 (연 2~4팀 → +2,000~5,000만원)</t>
         </is>
       </c>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="17" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1690,6 +1730,10 @@
           <t>• F-4 미국인 대표: 미국 현지 직접 수배로 중간 마진 제거 → 원가 절감 가능</t>
         </is>
       </c>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="17" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1697,6 +1741,10 @@
           <t>• 세금: 법인세 9% (과세표준 2억 이하)</t>
         </is>
       </c>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1736,6 +1784,10 @@
           <t>국내외여행업 → 종합여행업 전환 로드맵</t>
         </is>
       </c>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="17" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">

</xml_diff>